<commit_message>
up to v1_node_models.json is working
</commit_message>
<xml_diff>
--- a/V1model_seed_file.xlsx
+++ b/V1model_seed_file.xlsx
@@ -5,16 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shinya.ito/wsdata/network_builder/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shinya.ito/wsdata/glif_builder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B333CFB1-EEE1-E14C-A12E-92C5CF62E4A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46A49E66-3137-524E-A3E0-C8BC242B51B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-25600" yWindow="16960" windowWidth="25600" windowHeight="15540" activeTab="1" xr2:uid="{CFFEA874-25CC-4540-BE90-5AB415846019}"/>
   </bookViews>
   <sheets>
-    <sheet name="Number of cells in each layer" sheetId="1" r:id="rId1"/>
-    <sheet name="General Properties" sheetId="2" r:id="rId2"/>
+    <sheet name="cell_models" sheetId="1" r:id="rId1"/>
+    <sheet name="general_parameters" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>